<commit_message>
# [UI] Eliminar la sección «Ejemplos rápidos de prueba» de la interfaz Fixes #1
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Ferreteria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0790E895-23AA-4438-9DC6-77359CB89640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3861AF56-32B3-4F7E-8577-17074CD4E03F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -386,7 +386,7 @@
     <t>Verificar lectura de Excel, SKU, stock, rack/columna/fila, búsqueda, idioma, interfaz móvil y logs en la URL desplegada; no declarar éxito sin probar.</t>
   </si>
   <si>
-    <t>Martillo de peña1234567</t>
+    <t>Martillo de peña123</t>
   </si>
 </sst>
 </file>

</xml_diff>